<commit_message>
Edificios: alturas del Tejido Urbano por parcela y barrio, cruzadas con Parcelas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes_gemelo_buenos_aires.xlsx
+++ b/fuentes_gemelo_buenos_aires.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -990,7 +990,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Tipo de obra (acronimo/descripcion) por barrio; no hay superficie ni altura: no sirve para volúmenes 3D</t>
+          <t>Tipo de obra (acronimo/descripcion) por barrio; son permisos: las alturas vienen de ba_tejido_urbano</t>
         </is>
       </c>
     </row>
@@ -1000,27 +1000,27 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ba_presupuesto</t>
+          <t>ba_parcelas</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto Ejecutado 2026</t>
+          <t>Parcelas</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>municipio</t>
+          <t>edificios</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado-2026</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/parcelas</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Creative Commons Attribution</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1035,17 +1035,17 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2026, 2026-06</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>devengado_2026=7.672.722.979.847 pesos corrientes devengados (acumulado al T2); ejecucion_2026=36.7 % del crédito vigente devengado (acumulado al T2); registros=38.756 filas de presupuesto (2026 T2); sancionado_2026=18.189.401.033.591 pesos corrientes (crédito sancionado); vigente_2026=20.878.860.043.433 pesos corrientes (crédito vigente al T2)</t>
+          <t>parcelas_cruzadas_con_barrio=308.340 parcelas edificadas con barrio (por parcela o por manzana)</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Solo el último trimestre publicado (acumulado); falta ajuste por inflación y desglose por objeto del gasto</t>
+          <t>Solo se usa smp → barrio; geometría de parcelas (329 MB) no cargada</t>
         </is>
       </c>
     </row>
@@ -1055,12 +1055,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ba_presupuesto_historico</t>
+          <t>ba_presupuesto</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto Ejecutado</t>
+          <t>Presupuesto Ejecutado 2026</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1070,12 +1070,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado-2026</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-2.5-AR</t>
+          <t>Creative Commons Attribution</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2025, 2025-12</t>
+          <t>2026, 2026-06</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>devengado_2025=14.414.804.160.946 pesos corrientes devengados (año completo); vigente_2025=14.752.026.974.205 pesos corrientes (crédito vigente al cierre)</t>
+          <t>devengado_2026=7.672.722.979.847 pesos corrientes devengados (acumulado al T2); ejecucion_2026=36.7 % del crédito vigente devengado (acumulado al T2); registros=38.756 filas de presupuesto (2026 T2); sancionado_2026=18.189.401.033.591 pesos corrientes (crédito sancionado); vigente_2026=20.878.860.043.433 pesos corrientes (crédito vigente al T2)</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Solo el último año cerrado; 2013-2024 sin cargar (serie histórica en pesos corrientes)</t>
+          <t>Solo el último trimestre publicado (acumulado); falta ajuste por inflación y desglose por objeto del gasto</t>
         </is>
       </c>
     </row>
@@ -1110,22 +1110,22 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>ba_sensores_transito</t>
+          <t>ba_presupuesto_historico</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Sensores de Tránsito</t>
+          <t>Presupuesto Ejecutado</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>sensores</t>
+          <t>municipio</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/sensores-transito</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1145,17 +1145,17 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2025, 2025-12</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>ba_sensores_transito=52 sensores de tránsito</t>
+          <t>devengado_2025=14.414.804.160.946 pesos corrientes devengados (año completo); vigente_2025=14.752.026.974.205 pesos corrientes (crédito vigente al cierre)</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Lecturas en vivo (API de transporte con credenciales); aquí solo inventario de 52 sensores</t>
+          <t>Solo el último año cerrado; 2013-2024 sin cargar (serie histórica en pesos corrientes)</t>
         </is>
       </c>
     </row>
@@ -1165,22 +1165,22 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ba_subte_estaciones</t>
+          <t>ba_sensores_transito</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Subte: Estaciones.</t>
+          <t>Sensores de Tránsito</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>geoinfraestructura</t>
+          <t>sensores</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/subte-estaciones</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/sensores-transito</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1200,17 +1200,17 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>estaciones_distintas=88 estaciones (nombres distintos); estaciones_linea=90 pares estación-línea; lineas=6 líneas</t>
+          <t>ba_sensores_transito=52 sensores de tránsito</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Accesibilidad; campo línea (A, B, C…) en subte_lineas.geojson. Viajes por estación: ver ba_subte_molinetes</t>
+          <t>Lecturas en vivo (API de transporte con credenciales); aquí solo inventario de 52 sensores</t>
         </is>
       </c>
     </row>
@@ -1220,22 +1220,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>ba_subte_molinetes</t>
+          <t>ba_subte_estaciones</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Subte: Viajes Molinetes.</t>
+          <t>Subte: Estaciones.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>subte_molinetes</t>
+          <t>geoinfraestructura</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/subte-viajes-molinetes</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/subte-estaciones</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1255,17 +1255,17 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>lineas=7 líneas (incluye Premetro PM); meses_con_datos_2025=12 meses; pasajeros_subte_2025=206.459.041 pasajeros (validaciones en molinetes. líneas A-H)</t>
+          <t>estaciones_distintas=88 estaciones (nombres distintos); estaciones_linea=90 pares estación-línea; lineas=6 líneas</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Franja horaria (cada 15 min) y años anteriores sin cargar; se guarda solo el agregado por estación y mes</t>
+          <t>Accesibilidad; campo línea (A, B, C…) en subte_lineas.geojson. Viajes por estación: ver ba_subte_molinetes</t>
         </is>
       </c>
     </row>
@@ -1275,22 +1275,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>ba_tmi</t>
+          <t>ba_subte_molinetes</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Información Meteorológica</t>
+          <t>Subte: Viajes Molinetes.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>sensores</t>
+          <t>subte_molinetes</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-meteorologica</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/subte-viajes-molinetes</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1310,17 +1310,17 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>ba_tmi=16 torres de monitoreo inteligente</t>
+          <t>lineas=7 líneas (incluye Premetro PM); meses_con_datos_2025=12 meses; pasajeros_subte_2025=206.459.041 pasajeros (validaciones en molinetes. líneas A-H)</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Lecturas meteorológicas de las torres (temperatura, humedad); aquí solo inventario de 16 torres</t>
+          <t>Franja horaria (cada 15 min) y años anteriores sin cargar; se guarda solo el agregado por estación y mes</t>
         </is>
       </c>
     </row>
@@ -1330,32 +1330,32 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>dgeyc_censo2022</t>
+          <t>ba_tejido_urbano</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Censo Nacional 2022, resultados definitivos CABA (INDEC; DGEyC GCBA, informe 1877)</t>
+          <t>Tejido Urbano</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, demografia</t>
+          <t>edificios</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.estadisticaciudad.gob.ar/eyc/wp-content/uploads/2024/07/ir_2024_1877.pdf</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/tejido-urbano</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>sin licencia declarada (publicación oficial; citar fuente)</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>declarado</t>
+          <t>vivo</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1365,17 +1365,17 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>poblacion_comunas=3.121.707 habitantes (Censo 2022 definitivo. suma de comunas)</t>
+          <t>altura_maxima=221.4 m (volumen más alto del tejido); altura_mediana_parcela=5.6 m (mediana de la altura máxima por parcela); parcelas_edificadas=309.164 parcelas edificadas; volumenes_descartados=2 volúmenes con altura 0 o mayor a 250 m (errores); volumenes_edificados=1.386.616 volúmenes edificados (filas del tejido)</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Solo población por comuna. Faltan viviendas, hogares y servicios por comuna (informe 1877 los trae en gráficos) y radios censales</t>
+          <t>Superficie de cada volumen (para m³ construidos) y geometrías 3D (~1 GB: GeoParquet/PMTiles, ver contrato); datos hasta 2021</t>
         </is>
       </c>
     </row>
@@ -1385,27 +1385,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>eoh_caba</t>
+          <t>ba_tmi</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Encuesta de Ocupación Hotelera y Parahotelera (EOH), INDEC y Subsecretaría de Turismo</t>
+          <t>Información Meteorológica</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>turismo</t>
+          <t>sensores</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://datos.yvera.gob.ar/dataset/encuesta-ocupacion-hotelera-parahotelera-eoh</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-meteorologica</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1420,17 +1420,17 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2024, 2025-08</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>ocupacion_plazas_ultimo_mes=39.0 % de plazas ocupadas (hoteles y parahoteles); pernoctaciones_ultimo_mes=660.646 pernoctaciones (noches) por mes; viajeros_2024=3.993.697 viajeros hospedados en el año; viajeros_no_residentes_ultimo_mes=136.364 viajeros no residentes hospedados por mes; viajeros_residentes_ultimo_mes=173.564 viajeros residentes hospedados por mes; viajeros_total_ultimo_mes=309.928 viajeros hospedados por mes</t>
+          <t>ba_tmi=16 torres de monitoreo inteligente</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Tarifa media, estadía media y ocupación por categoría; se publica con ~1 año de rezago</t>
+          <t>Lecturas meteorológicas de las torres (temperatura, humedad); aquí solo inventario de 16 torres</t>
         </is>
       </c>
     </row>
@@ -1440,32 +1440,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>wikimedia_pageviews</t>
+          <t>dgeyc_censo2022</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Wikimedia Pageviews API</t>
+          <t>Censo Nacional 2022, resultados definitivos CABA (INDEC; DGEyC GCBA, informe 1877)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>escucha</t>
+          <t>correlaciones, demografia</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://wikimedia.org/api/rest_v1/metrics/pageviews/per-article/es.wikipedia/all-access/user/Buenos_Aires/monthly/20250101/20260831</t>
+          <t>https://www.estadisticaciudad.gob.ar/eyc/wp-content/uploads/2024/07/ir_2024_1877.pdf</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>CC0</t>
+          <t>sin licencia declarada (publicación oficial; citar fuente)</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>vivo</t>
+          <t>declarado</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1475,17 +1475,17 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>vistas_ultimo_mes=36.339 vistas de personas</t>
+          <t>poblacion_comunas=3.121.707 habitantes (Censo 2022 definitivo. suma de comunas)</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Otros artículos/idiomas; mide interés, no opinión ni sentimiento</t>
+          <t>Solo población por comuna. Faltan viviendas, hogares y servicios por comuna (informe 1877 los trae en gráficos) y radios censales</t>
         </is>
       </c>
     </row>
@@ -1493,38 +1493,54 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>eoh_caba</t>
+        </is>
+      </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Tejido Urbano (BA Data, Secretaría de Desarrollo Urbano)</t>
+          <t>Encuesta de Ocupación Hotelera y Parahotelera (EOH), INDEC y Subsecretaría de Turismo</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>(edificios 3D)</t>
+          <t>turismo</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/tejido-urbano</t>
+          <t>https://datos.yvera.gob.ar/dataset/encuesta-ocupacion-hotelera-parahotelera-eoh</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-2.5-AR</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>identificado</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr"/>
-      <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="2" t="inlineStr"/>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>2024, 2025-08</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>ocupacion_plazas_ultimo_mes=39.0 % de plazas ocupadas (hoteles y parahoteles); pernoctaciones_ultimo_mes=660.646 pernoctaciones (noches) por mes; viajeros_2024=3.993.697 viajeros hospedados en el año; viajeros_no_residentes_ultimo_mes=136.364 viajeros no residentes hospedados por mes; viajeros_residentes_ultimo_mes=173.564 viajeros residentes hospedados por mes; viajeros_total_ultimo_mes=309.928 viajeros hospedados por mes</t>
+        </is>
+      </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Alturas (m) y pisos por volumen edificado, datos hasta 2021. GeoJSON 1,09 GB y CSV 122 MB: no cabe en GeoJSON simplificado, pasa a GeoParquet/PMTiles (ver contrato). Por barrio requiere cruzar con Parcelas (329 MB) por smp</t>
+          <t>Tarifa media, estadía media y ocupación por categoría; se publica con ~1 año de rezago</t>
         </is>
       </c>
     </row>
@@ -1532,38 +1548,54 @@
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>wikimedia_pageviews</t>
+        </is>
+      </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Información Censal por Radio (BA Data)</t>
+          <t>Wikimedia Pageviews API</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>(demografía 2022 por barrio)</t>
+          <t>escucha</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-censal-por-radio</t>
+          <t>https://wikimedia.org/api/rest_v1/metrics/pageviews/per-article/es.wikipedia/all-access/user/Buenos_Aires/monthly/20250101/20260831</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-2.5-AR</t>
+          <t>CC0</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>insuficiente</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
-      <c r="I21" s="2" t="inlineStr"/>
-      <c r="J21" s="2" t="inlineStr"/>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>vistas_ultimo_mes=36.339 vistas de personas</t>
+        </is>
+      </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Solo radios de 2001 y 2010: no da población 2022 por barrio. Los radios 2022 no están en BA Data</t>
+          <t>Otros artículos/idiomas; mide interés, no opinión ni sentimiento</t>
         </is>
       </c>
     </row>
@@ -1574,19 +1606,27 @@
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>BA Data reclamos 147</t>
+          <t>Información Censal por Radio (BA Data)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>(reclamos)</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
+          <t>(demografía 2022 por barrio)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-censal-por-radio</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>CC-BY-2.5-AR</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>descartado</t>
+          <t>insuficiente</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -1594,7 +1634,7 @@
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Descartado por descarga pesada; faltan todos los campos</t>
+          <t>Solo radios de 2001 y 2010: no da población 2022 por barrio. Los radios 2022 no están en BA Data</t>
         </is>
       </c>
     </row>
@@ -1605,19 +1645,19 @@
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>API de transporte/sensores</t>
+          <t>BA Data reclamos 147</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>(sensores en tiempo real)</t>
+          <t>(reclamos)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>pendiente</t>
+          <t>descartado</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1625,6 +1665,37 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr">
         <is>
+          <t>Descartado por descarga pesada; faltan todos los campos</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>API de transporte/sensores</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>(sensores en tiempo real)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>pendiente</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
           <t>Requiere credenciales; faltan lecturas, frecuencia y licencia</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Tres fuentes nuevas: espacios verdes, establecimientos educativos y hospitales (23 fuentes vivas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes_gemelo_buenos_aires.xlsx
+++ b/fuentes_gemelo_buenos_aires.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -945,22 +945,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ba_obras_registradas</t>
+          <t>ba_espacios_verdes</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Obras Registradas</t>
+          <t>Espacios Verdes</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, edificios</t>
+          <t>espacios_verdes</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/obras-registradas</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/espacios-verdes</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -980,17 +980,17 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>registros=87.784 obras registradas</t>
+          <t>registros=2.176 espacios verdes públicos; superficie_m2=15.838.266 m² de espacio verde público</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Tipo de obra (acronimo/descripcion) por barrio; son permisos: las alturas vienen de ba_tejido_urbano</t>
+          <t>Arbolado; espacios verdes privados; m² por habitante (población 2022 por barrio no disponible)</t>
         </is>
       </c>
     </row>
@@ -1000,22 +1000,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ba_parcelas</t>
+          <t>ba_establecimientos_educativos</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Parcelas</t>
+          <t>Establecimientos Educativos</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>edificios</t>
+          <t>educacion</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/parcelas</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/establecimientos-educativos</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1035,17 +1035,17 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>parcelas_cruzadas_con_barrio=308.340 parcelas edificadas con barrio (por parcela o por manzana)</t>
+          <t>estatales=1.773 establecimientos de gestión estatal; registros=2.767 establecimientos educativos (oferta por nivel)</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Solo se usa smp → barrio; geometría de parcelas (329 MB) no cargada</t>
+          <t>Matrícula (alumnos) y cargos docentes; el padrón trae correos y no se usa</t>
         </is>
       </c>
     </row>
@@ -1055,27 +1055,27 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ba_presupuesto</t>
+          <t>ba_hospitales</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto Ejecutado 2026</t>
+          <t>Hospitales</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>municipio</t>
+          <t>salud</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado-2026</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/hospitales</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Creative Commons Attribution</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026, 2026-06</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>devengado_2026=7.672.722.979.847 pesos corrientes devengados (acumulado al T2); ejecucion_2026=36.7 % del crédito vigente devengado (acumulado al T2); registros=38.756 filas de presupuesto (2026 T2); sancionado_2026=18.189.401.033.591 pesos corrientes (crédito sancionado); vigente_2026=20.878.860.043.433 pesos corrientes (crédito vigente al T2)</t>
+          <t>registros=36 hospitales públicos</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Solo el último trimestre publicado (acumulado); falta ajuste por inflación y desglose por objeto del gasto</t>
+          <t>Camas, egresos y guardias (otros conjuntos: movimiento hospitalario); CESAC y privados no incluidos</t>
         </is>
       </c>
     </row>
@@ -1110,22 +1110,22 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>ba_presupuesto_historico</t>
+          <t>ba_obras_registradas</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto Ejecutado</t>
+          <t>Obras Registradas</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>municipio</t>
+          <t>correlaciones, edificios</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/obras-registradas</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1145,17 +1145,17 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2025, 2025-12</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>devengado_2025=14.414.804.160.946 pesos corrientes devengados (año completo); vigente_2025=14.752.026.974.205 pesos corrientes (crédito vigente al cierre)</t>
+          <t>registros=87.784 obras registradas</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Solo el último año cerrado; 2013-2024 sin cargar (serie histórica en pesos corrientes)</t>
+          <t>Tipo de obra (acronimo/descripcion) por barrio; son permisos: las alturas vienen de ba_tejido_urbano</t>
         </is>
       </c>
     </row>
@@ -1165,22 +1165,22 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ba_sensores_transito</t>
+          <t>ba_parcelas</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Sensores de Tránsito</t>
+          <t>Parcelas</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>sensores</t>
+          <t>correlaciones, edificios</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/sensores-transito</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/parcelas</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1200,17 +1200,17 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>ba_sensores_transito=52 sensores de tránsito</t>
+          <t>parcelas_cruzadas_con_barrio=308.340 parcelas edificadas con barrio (por parcela o por manzana)</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Lecturas en vivo (API de transporte con credenciales); aquí solo inventario de 52 sensores</t>
+          <t>Solo se usa smp → barrio; geometría de parcelas (329 MB) no cargada</t>
         </is>
       </c>
     </row>
@@ -1220,27 +1220,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>ba_subte_estaciones</t>
+          <t>ba_presupuesto</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Subte: Estaciones.</t>
+          <t>Presupuesto Ejecutado 2026</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>geoinfraestructura</t>
+          <t>municipio</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/subte-estaciones</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado-2026</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-2.5-AR</t>
+          <t>Creative Commons Attribution</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1255,17 +1255,17 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026, 2026-06</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>estaciones_distintas=88 estaciones (nombres distintos); estaciones_linea=90 pares estación-línea; lineas=6 líneas</t>
+          <t>devengado_2026=7.672.722.979.847 pesos corrientes devengados (acumulado al T2); ejecucion_2026=36.7 % del crédito vigente devengado (acumulado al T2); registros=38.756 filas de presupuesto (2026 T2); sancionado_2026=18.189.401.033.591 pesos corrientes (crédito sancionado); vigente_2026=20.878.860.043.433 pesos corrientes (crédito vigente al T2)</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Accesibilidad; campo línea (A, B, C…) en subte_lineas.geojson. Viajes por estación: ver ba_subte_molinetes</t>
+          <t>Solo el último trimestre publicado (acumulado); falta ajuste por inflación y desglose por objeto del gasto</t>
         </is>
       </c>
     </row>
@@ -1275,22 +1275,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>ba_subte_molinetes</t>
+          <t>ba_presupuesto_historico</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Subte: Viajes Molinetes.</t>
+          <t>Presupuesto Ejecutado</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>subte_molinetes</t>
+          <t>municipio</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/subte-viajes-molinetes</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1310,17 +1310,17 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025, 2025-12</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>lineas=7 líneas (incluye Premetro PM); meses_con_datos_2025=12 meses; pasajeros_subte_2025=206.459.041 pasajeros (validaciones en molinetes. líneas A-H)</t>
+          <t>devengado_2025=14.414.804.160.946 pesos corrientes devengados (año completo); vigente_2025=14.752.026.974.205 pesos corrientes (crédito vigente al cierre)</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Franja horaria (cada 15 min) y años anteriores sin cargar; se guarda solo el agregado por estación y mes</t>
+          <t>Solo el último año cerrado; 2013-2024 sin cargar (serie histórica en pesos corrientes)</t>
         </is>
       </c>
     </row>
@@ -1330,22 +1330,22 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>ba_tejido_urbano</t>
+          <t>ba_sensores_transito</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Tejido Urbano</t>
+          <t>Sensores de Tránsito</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>edificios</t>
+          <t>sensores</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/tejido-urbano</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/sensores-transito</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1365,17 +1365,17 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>altura_maxima=221.4 m (volumen más alto del tejido); altura_mediana_parcela=5.6 m (mediana de la altura máxima por parcela); parcelas_edificadas=309.164 parcelas edificadas; volumenes_descartados=2 volúmenes con altura 0 o mayor a 250 m (errores); volumenes_edificados=1.386.616 volúmenes edificados (filas del tejido)</t>
+          <t>ba_sensores_transito=52 sensores de tránsito</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Superficie de cada volumen (para m³ construidos) y geometrías 3D (~1 GB: GeoParquet/PMTiles, ver contrato); datos hasta 2021</t>
+          <t>Lecturas en vivo (API de transporte con credenciales); aquí solo inventario de 52 sensores</t>
         </is>
       </c>
     </row>
@@ -1385,22 +1385,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ba_tmi</t>
+          <t>ba_subte_estaciones</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Información Meteorológica</t>
+          <t>Subte: Estaciones.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>sensores</t>
+          <t>geoinfraestructura</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-meteorologica</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/subte-estaciones</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1420,17 +1420,17 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>ba_tmi=16 torres de monitoreo inteligente</t>
+          <t>estaciones_distintas=88 estaciones (nombres distintos); estaciones_linea=90 pares estación-línea; lineas=6 líneas</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Lecturas meteorológicas de las torres (temperatura, humedad); aquí solo inventario de 16 torres</t>
+          <t>Accesibilidad; campo línea (A, B, C…) en subte_lineas.geojson. Viajes por estación: ver ba_subte_molinetes</t>
         </is>
       </c>
     </row>
@@ -1440,32 +1440,32 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>dgeyc_censo2022</t>
+          <t>ba_subte_molinetes</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Censo Nacional 2022, resultados definitivos CABA (INDEC; DGEyC GCBA, informe 1877)</t>
+          <t>Subte: Viajes Molinetes.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, demografia</t>
+          <t>subte_molinetes</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.estadisticaciudad.gob.ar/eyc/wp-content/uploads/2024/07/ir_2024_1877.pdf</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/subte-viajes-molinetes</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>sin licencia declarada (publicación oficial; citar fuente)</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>declarado</t>
+          <t>vivo</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1475,17 +1475,17 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>poblacion_comunas=3.121.707 habitantes (Censo 2022 definitivo. suma de comunas)</t>
+          <t>lineas=7 líneas (incluye Premetro PM); meses_con_datos_2025=12 meses; pasajeros_subte_2025=206.459.041 pasajeros (validaciones en molinetes. líneas A-H)</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Solo población por comuna. Faltan viviendas, hogares y servicios por comuna (informe 1877 los trae en gráficos) y radios censales</t>
+          <t>Franja horaria (cada 15 min) y años anteriores sin cargar; se guarda solo el agregado por estación y mes</t>
         </is>
       </c>
     </row>
@@ -1495,27 +1495,27 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>eoh_caba</t>
+          <t>ba_tejido_urbano</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Encuesta de Ocupación Hotelera y Parahotelera (EOH), INDEC y Subsecretaría de Turismo</t>
+          <t>Tejido Urbano</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>turismo</t>
+          <t>correlaciones, edificios</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://datos.yvera.gob.ar/dataset/encuesta-ocupacion-hotelera-parahotelera-eoh</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/tejido-urbano</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1530,17 +1530,17 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2024, 2025-08</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>ocupacion_plazas_ultimo_mes=39.0 % de plazas ocupadas (hoteles y parahoteles); pernoctaciones_ultimo_mes=660.646 pernoctaciones (noches) por mes; viajeros_2024=3.993.697 viajeros hospedados en el año; viajeros_no_residentes_ultimo_mes=136.364 viajeros no residentes hospedados por mes; viajeros_residentes_ultimo_mes=173.564 viajeros residentes hospedados por mes; viajeros_total_ultimo_mes=309.928 viajeros hospedados por mes</t>
+          <t>altura_maxima=221.4 m (volumen más alto del tejido); altura_mediana_parcela=5.6 m (mediana de la altura máxima por parcela); parcelas_edificadas=309.164 parcelas edificadas; volumenes_descartados=2 volúmenes con altura 0 o mayor a 250 m (errores); volumenes_edificados=1.386.616 volúmenes edificados (filas del tejido)</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Tarifa media, estadía media y ocupación por categoría; se publica con ~1 año de rezago</t>
+          <t>Superficie de cada volumen (para m³ construidos) y geometrías 3D (~1 GB: GeoParquet/PMTiles, ver contrato); datos hasta 2021</t>
         </is>
       </c>
     </row>
@@ -1550,27 +1550,27 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>wikimedia_pageviews</t>
+          <t>ba_tmi</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Wikimedia Pageviews API</t>
+          <t>Información Meteorológica</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>escucha</t>
+          <t>sensores</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://wikimedia.org/api/rest_v1/metrics/pageviews/per-article/es.wikipedia/all-access/user/Buenos_Aires/monthly/20250101/20260831</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-meteorologica</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>CC0</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1585,17 +1585,17 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>vistas_ultimo_mes=36.339 vistas de personas</t>
+          <t>ba_tmi=16 torres de monitoreo inteligente</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Otros artículos/idiomas; mide interés, no opinión ni sentimiento</t>
+          <t>Lecturas meteorológicas de las torres (temperatura, humedad); aquí solo inventario de 16 torres</t>
         </is>
       </c>
     </row>
@@ -1603,38 +1603,54 @@
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>dgeyc_censo2022</t>
+        </is>
+      </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Información Censal por Radio (BA Data)</t>
+          <t>Censo Nacional 2022, resultados definitivos CABA (INDEC; DGEyC GCBA, informe 1877)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>(demografía 2022 por barrio)</t>
+          <t>correlaciones, demografia</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-censal-por-radio</t>
+          <t>https://www.estadisticaciudad.gob.ar/eyc/wp-content/uploads/2024/07/ir_2024_1877.pdf</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-2.5-AR</t>
+          <t>sin licencia declarada (publicación oficial; citar fuente)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>insuficiente</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="2" t="inlineStr"/>
+          <t>declarado</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>poblacion_comunas=3.121.707 habitantes (Censo 2022 definitivo. suma de comunas)</t>
+        </is>
+      </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Solo radios de 2001 y 2010: no da población 2022 por barrio. Los radios 2022 no están en BA Data</t>
+          <t>Solo población por comuna. Faltan viviendas, hogares y servicios por comuna (informe 1877 los trae en gráficos) y radios censales</t>
         </is>
       </c>
     </row>
@@ -1642,30 +1658,54 @@
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>eoh_caba</t>
+        </is>
+      </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>BA Data reclamos 147</t>
+          <t>Encuesta de Ocupación Hotelera y Parahotelera (EOH), INDEC y Subsecretaría de Turismo</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>(reclamos)</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
+          <t>turismo</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://datos.yvera.gob.ar/dataset/encuesta-ocupacion-hotelera-parahotelera-eoh</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>descartado</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>2024, 2025-08</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>ocupacion_plazas_ultimo_mes=39.0 % de plazas ocupadas (hoteles y parahoteles); pernoctaciones_ultimo_mes=660.646 pernoctaciones (noches) por mes; viajeros_2024=3.993.697 viajeros hospedados en el año; viajeros_no_residentes_ultimo_mes=136.364 viajeros no residentes hospedados por mes; viajeros_residentes_ultimo_mes=173.564 viajeros residentes hospedados por mes; viajeros_total_ultimo_mes=309.928 viajeros hospedados por mes</t>
+        </is>
+      </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Descartado por descarga pesada; faltan todos los campos</t>
+          <t>Tarifa media, estadía media y ocupación por categoría; se publica con ~1 año de rezago</t>
         </is>
       </c>
     </row>
@@ -1673,28 +1713,153 @@
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>wikimedia_pageviews</t>
+        </is>
+      </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
+          <t>Wikimedia Pageviews API</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>escucha</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://wikimedia.org/api/rest_v1/metrics/pageviews/per-article/es.wikipedia/all-access/user/Buenos_Aires/monthly/20250101/20260831</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>CC0</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>vistas_ultimo_mes=36.339 vistas de personas</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Otros artículos/idiomas; mide interés, no opinión ni sentimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Información Censal por Radio (BA Data)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>(demografía 2022 por barrio)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-censal-por-radio</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>CC-BY-2.5-AR</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>insuficiente</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>Solo radios de 2001 y 2010: no da población 2022 por barrio. Los radios 2022 no están en BA Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>BA Data reclamos 147</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>(reclamos)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>descartado</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Descartado por descarga pesada; faltan todos los campos</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
           <t>API de transporte/sensores</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>(sensores en tiempo real)</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>pendiente</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>Requiere credenciales; faltan lecturas, frecuencia y licencia</t>
         </is>

</xml_diff>

<commit_message>
Molinetes cruzados con la capa de estaciones y barrios; correlaciones con verde, escuelas, alturas y subte
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes_gemelo_buenos_aires.xlsx
+++ b/fuentes_gemelo_buenos_aires.xlsx
@@ -875,7 +875,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>barrios_comparados=48 barrios con todas las variables; poblacion_barrios=2.890.151 habitantes (Censo 2010. suma de barrios)</t>
+          <t>barrios_comparados=48 barrios con población y área; pares_fuertes=10 pares de indicadores con |Spearman| ≥ 0.5; poblacion_barrios=2.890.151 habitantes (Censo 2010. suma de barrios)</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>espacios_verdes</t>
+          <t>correlaciones, espacios_verdes</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>educacion</t>
+          <t>correlaciones, educacion</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>subte_molinetes</t>
+          <t>correlaciones, subte_molinetes</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, demografia</t>
+          <t>demografia</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Siete fuentes nuevas (30 vivas): IPCBA, SIPA, Open-Meteo, CESAC, EcoBici, paradas de colectivo y puntos verdes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes_gemelo_buenos_aires.xlsx
+++ b/fuentes_gemelo_buenos_aires.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -670,22 +670,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ba_comunas</t>
+          <t>ba_cesac</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Comunas</t>
+          <t>Centros de Salud y Acción Comunitaria (CESAC)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>atlas_zonas</t>
+          <t>salud</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/comunas</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/centros-salud-accion-comunitaria-cesac</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -705,17 +705,17 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>registros=15 comunas</t>
+          <t>cesac=50 Centros de Salud y Acción Comunitaria</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Densidad 2022 (cruzar con censo). Geometría en lago/geo/comunas.geojson</t>
+          <t>Especialidades por CESAC (campo especialid sin agregar); atenciones; teléfono/web no se copian</t>
         </is>
       </c>
     </row>
@@ -725,27 +725,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ba_data_ckan</t>
+          <t>ba_colectivos_paradas</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>BA Data (CKAN)</t>
+          <t>Colectivos: paradas</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>catalogo</t>
+          <t>movilidad</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/api/3/action/package_search?rows=1000</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/colectivos-paradas</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>por conjunto (ver licencia de cada uno)</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -760,17 +760,17 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>conjuntos=455 conjuntos de datos</t>
+          <t>lineas_colectivo=132 líneas de colectivo distintas con parada; paradas_colectivo=7.027 paradas de colectivo</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Ninguno: catálogo completo (455 conjuntos); falta monitorear cambios de licencia/actualización</t>
+          <t>Recorridos y frecuencias (GTFS); pasajeros por línea</t>
         </is>
       </c>
     </row>
@@ -780,27 +780,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ba_delitos</t>
+          <t>ba_comunas</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Delitos</t>
+          <t>Comunas</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, seguridad</t>
+          <t>atlas_zonas</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/delitos</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/comunas</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Creative Commons Attribution</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -815,17 +815,17 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>2024, 2025</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>delitos_2024=158.838 delitos registrados; delitos_2025=133.203 delitos registrados; meses_con_datos_2024=12 meses; meses_con_datos_2025=12 meses</t>
+          <t>registros=15 comunas</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Tasa por 1.000 hab, franja horaria, subtipo, uso de arma; años 2016-2023 sin cargar</t>
+          <t>Densidad 2022 (cruzar con censo). Geometría en lago/geo/comunas.geojson</t>
         </is>
       </c>
     </row>
@@ -835,27 +835,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ba_demografia</t>
+          <t>ba_data_ckan</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Estructura demográfica</t>
+          <t>BA Data (CKAN)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, demografia</t>
+          <t>catalogo</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/estructura-demografica</t>
+          <t>https://data.buenosaires.gob.ar/km/api/3/action/package_search?rows=1000</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-2.5-AR</t>
+          <t>por conjunto (ver licencia de cada uno)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -870,17 +870,17 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>2010, 2022, 2024</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>barrios_comparados=48 barrios con población y área; pares_fuertes=10 pares de indicadores con |Spearman| ≥ 0.5; poblacion_barrios=2.890.151 habitantes (Censo 2010. suma de barrios)</t>
+          <t>conjuntos=455 conjuntos de datos</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Edad y sexo por barrio, hogares, esperanza de vida (recursos del paquete sin curar); barrios aún Censo 2010</t>
+          <t>Ninguno: catálogo completo (455 conjuntos); falta monitorear cambios de licencia/actualización</t>
         </is>
       </c>
     </row>
@@ -890,27 +890,27 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ba_espacios_culturales</t>
+          <t>ba_delitos</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Espacios culturales.</t>
+          <t>Delitos</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, cultura</t>
+          <t>correlaciones, seguridad</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/espacios-culturales</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/delitos</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-2.5-AR</t>
+          <t>Creative Commons Attribution</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -925,17 +925,17 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2024, 2025</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>registros=3.053 espacios culturales</t>
+          <t>delitos_2024=158.838 delitos registrados; delitos_2025=133.203 delitos registrados; meses_con_datos_2024=12 meses; meses_con_datos_2025=12 meses</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Capacidad total y cantidad de salas por barrio (campos existen, no agregados); coordenadas no guardadas</t>
+          <t>Tasa por 1.000 hab, franja horaria, subtipo, uso de arma; años 2016-2023 sin cargar</t>
         </is>
       </c>
     </row>
@@ -945,22 +945,22 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>ba_espacios_verdes</t>
+          <t>ba_demografia</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Espacios Verdes</t>
+          <t>Estructura demográfica</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, espacios_verdes</t>
+          <t>correlaciones, demografia</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/espacios-verdes</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/estructura-demografica</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -980,17 +980,17 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2010, 2022, 2024</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>registros=2.176 espacios verdes públicos; superficie_m2=15.838.266 m² de espacio verde público</t>
+          <t>barrios_comparados=48 barrios con población y área; pares_fuertes=10 pares de indicadores con |Spearman| ≥ 0.5; poblacion_barrios=2.890.151 habitantes (Censo 2010. suma de barrios)</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Arbolado; espacios verdes privados; m² por habitante (población 2022 por barrio no disponible)</t>
+          <t>Edad y sexo por barrio, hogares, esperanza de vida (recursos del paquete sin curar); barrios aún Censo 2010</t>
         </is>
       </c>
     </row>
@@ -1000,22 +1000,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>ba_establecimientos_educativos</t>
+          <t>ba_ecobici_estaciones</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Establecimientos Educativos</t>
+          <t>Estaciones Bicicletas Públicas.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, educacion</t>
+          <t>movilidad</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/establecimientos-educativos</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/estaciones-bicicletas-publicas</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1040,12 +1040,12 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>estatales=1.773 establecimientos de gestión estatal; registros=2.767 establecimientos educativos (oferta por nivel)</t>
+          <t>estaciones_ecobici=407 estaciones de bicicletas públicas</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Matrícula (alumnos) y cargos docentes; el padrón trae correos y no se usa</t>
+          <t>Viajes en EcoBici (conjunto bicicletas-publicas, pesado) y capacidad de anclajes</t>
         </is>
       </c>
     </row>
@@ -1055,22 +1055,22 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>ba_hospitales</t>
+          <t>ba_espacios_culturales</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Hospitales</t>
+          <t>Espacios culturales.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>salud</t>
+          <t>correlaciones, cultura</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/hospitales</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/espacios-culturales</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1090,17 +1090,17 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-06</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>registros=36 hospitales públicos</t>
+          <t>registros=3.053 espacios culturales</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Camas, egresos y guardias (otros conjuntos: movimiento hospitalario); CESAC y privados no incluidos</t>
+          <t>Capacidad total y cantidad de salas por barrio (campos existen, no agregados); coordenadas no guardadas</t>
         </is>
       </c>
     </row>
@@ -1110,22 +1110,22 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>ba_obras_registradas</t>
+          <t>ba_espacios_verdes</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Obras Registradas</t>
+          <t>Espacios Verdes</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, edificios</t>
+          <t>correlaciones, espacios_verdes</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/obras-registradas</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/espacios-verdes</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1145,17 +1145,17 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>registros=87.784 obras registradas</t>
+          <t>registros=2.176 espacios verdes públicos; superficie_m2=15.838.266 m² de espacio verde público</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Tipo de obra (acronimo/descripcion) por barrio; son permisos: las alturas vienen de ba_tejido_urbano</t>
+          <t>Arbolado; espacios verdes privados; m² por habitante (población 2022 por barrio no disponible)</t>
         </is>
       </c>
     </row>
@@ -1165,22 +1165,22 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>ba_parcelas</t>
+          <t>ba_establecimientos_educativos</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Parcelas</t>
+          <t>Establecimientos Educativos</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, edificios</t>
+          <t>correlaciones, educacion</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/parcelas</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/establecimientos-educativos</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1200,17 +1200,17 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>parcelas_cruzadas_con_barrio=308.340 parcelas edificadas con barrio (por parcela o por manzana)</t>
+          <t>estatales=1.773 establecimientos de gestión estatal; registros=2.767 establecimientos educativos (oferta por nivel)</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Solo se usa smp → barrio; geometría de parcelas (329 MB) no cargada</t>
+          <t>Matrícula (alumnos) y cargos docentes; el padrón trae correos y no se usa</t>
         </is>
       </c>
     </row>
@@ -1220,27 +1220,27 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>ba_presupuesto</t>
+          <t>ba_hospitales</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto Ejecutado 2026</t>
+          <t>Hospitales</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>municipio</t>
+          <t>salud</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado-2026</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/hospitales</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Creative Commons Attribution</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1255,17 +1255,17 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>2026, 2026-06</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>devengado_2026=7.672.722.979.847 pesos corrientes devengados (acumulado al T2); ejecucion_2026=36.7 % del crédito vigente devengado (acumulado al T2); registros=38.756 filas de presupuesto (2026 T2); sancionado_2026=18.189.401.033.591 pesos corrientes (crédito sancionado); vigente_2026=20.878.860.043.433 pesos corrientes (crédito vigente al T2)</t>
+          <t>registros=36 hospitales públicos</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Solo el último trimestre publicado (acumulado); falta ajuste por inflación y desglose por objeto del gasto</t>
+          <t>Camas, egresos y guardias (otros conjuntos: movimiento hospitalario); CESAC y privados no incluidos</t>
         </is>
       </c>
     </row>
@@ -1275,22 +1275,22 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>ba_presupuesto_historico</t>
+          <t>ba_obras_registradas</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Presupuesto Ejecutado</t>
+          <t>Obras Registradas</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>municipio</t>
+          <t>correlaciones, edificios</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/obras-registradas</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1310,17 +1310,17 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>2025, 2025-12</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>devengado_2025=14.414.804.160.946 pesos corrientes devengados (año completo); vigente_2025=14.752.026.974.205 pesos corrientes (crédito vigente al cierre)</t>
+          <t>registros=87.784 obras registradas</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Solo el último año cerrado; 2013-2024 sin cargar (serie histórica en pesos corrientes)</t>
+          <t>Tipo de obra (acronimo/descripcion) por barrio; son permisos: las alturas vienen de ba_tejido_urbano</t>
         </is>
       </c>
     </row>
@@ -1330,22 +1330,22 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>ba_sensores_transito</t>
+          <t>ba_parcelas</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Sensores de Tránsito</t>
+          <t>Parcelas</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>sensores</t>
+          <t>correlaciones, edificios</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/sensores-transito</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/parcelas</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1365,17 +1365,17 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>ba_sensores_transito=52 sensores de tránsito</t>
+          <t>parcelas_cruzadas_con_barrio=308.340 parcelas edificadas con barrio (por parcela o por manzana)</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Lecturas en vivo (API de transporte con credenciales); aquí solo inventario de 52 sensores</t>
+          <t>Solo se usa smp → barrio; geometría de parcelas (329 MB) no cargada</t>
         </is>
       </c>
     </row>
@@ -1385,27 +1385,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>ba_subte_estaciones</t>
+          <t>ba_presupuesto</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Subte: Estaciones.</t>
+          <t>Presupuesto Ejecutado 2026</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>geoinfraestructura</t>
+          <t>municipio</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/subte-estaciones</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado-2026</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-2.5-AR</t>
+          <t>Creative Commons Attribution</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1420,17 +1420,17 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026, 2026-06</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>estaciones_distintas=88 estaciones (nombres distintos); estaciones_linea=90 pares estación-línea; lineas=6 líneas</t>
+          <t>devengado_2026=7.672.722.979.847 pesos corrientes devengados (acumulado al T2); ejecucion_2026=36.7 % del crédito vigente devengado (acumulado al T2); registros=38.756 filas de presupuesto (2026 T2); sancionado_2026=18.189.401.033.591 pesos corrientes (crédito sancionado); vigente_2026=20.878.860.043.433 pesos corrientes (crédito vigente al T2)</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Accesibilidad; campo línea (A, B, C…) en subte_lineas.geojson. Viajes por estación: ver ba_subte_molinetes</t>
+          <t>Solo el último trimestre publicado (acumulado); falta ajuste por inflación y desglose por objeto del gasto</t>
         </is>
       </c>
     </row>
@@ -1440,22 +1440,22 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>ba_subte_molinetes</t>
+          <t>ba_presupuesto_historico</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Subte: Viajes Molinetes.</t>
+          <t>Presupuesto Ejecutado</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, subte_molinetes</t>
+          <t>municipio</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/subte-viajes-molinetes</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/presupuesto-ejecutado</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1475,17 +1475,17 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2025, 2025-12</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>lineas=7 líneas (incluye Premetro PM); meses_con_datos_2025=12 meses; pasajeros_subte_2025=206.459.041 pasajeros (validaciones en molinetes. líneas A-H)</t>
+          <t>devengado_2025=14.414.804.160.946 pesos corrientes devengados (año completo); devengado_2025_a_precios_2026-08=19.737.444.133.889 pesos de 2026-08 (devengado 2025 × IPCBA 2026-08 / IPCBA promedio 2025); vigente_2025=14.752.026.974.205 pesos corrientes (crédito vigente al cierre)</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Franja horaria (cada 15 min) y años anteriores sin cargar; se guarda solo el agregado por estación y mes</t>
+          <t>Solo el último año cerrado; 2013-2024 sin cargar (serie histórica en pesos corrientes)</t>
         </is>
       </c>
     </row>
@@ -1495,22 +1495,22 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ba_tejido_urbano</t>
+          <t>ba_puntos_verdes</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Tejido Urbano</t>
+          <t>Gestión de Residuos en Puntos Verdes</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>correlaciones, edificios</t>
+          <t>residuos</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/tejido-urbano</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/puntos-verdes</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1530,17 +1530,17 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2025, 2026-10</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>altura_maxima=221.4 m (volumen más alto del tejido); altura_mediana_parcela=5.6 m (mediana de la altura máxima por parcela); parcelas_edificadas=309.164 parcelas edificadas; volumenes_descartados=2 volúmenes con altura 0 o mayor a 250 m (errores); volumenes_edificados=1.386.616 volúmenes edificados (filas del tejido)</t>
+          <t>puntos_verdes=17 puntos verdes; raee_kg_2025=57.040 kg de RAEE recibidos en el año</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Superficie de cada volumen (para m³ construidos) y geometrías 3D (~1 GB: GeoParquet/PMTiles, ver contrato); datos hasta 2021</t>
+          <t>Materiales recibidos por punto (pesajes 2015-2019); el listado solo trae 17 puntos con atención</t>
         </is>
       </c>
     </row>
@@ -1550,12 +1550,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ba_tmi</t>
+          <t>ba_sensores_transito</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Información Meteorológica</t>
+          <t>Sensores de Tránsito</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-meteorologica</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/sensores-transito</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1590,12 +1590,12 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>ba_tmi=16 torres de monitoreo inteligente</t>
+          <t>ba_sensores_transito=52 sensores de tránsito</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Lecturas meteorológicas de las torres (temperatura, humedad); aquí solo inventario de 16 torres</t>
+          <t>Lecturas en vivo (API de transporte con credenciales); aquí solo inventario de 52 sensores</t>
         </is>
       </c>
     </row>
@@ -1605,32 +1605,32 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>dgeyc_censo2022</t>
+          <t>ba_subte_estaciones</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Censo Nacional 2022, resultados definitivos CABA (INDEC; DGEyC GCBA, informe 1877)</t>
+          <t>Subte: Estaciones.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>demografia</t>
+          <t>geoinfraestructura</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.estadisticaciudad.gob.ar/eyc/wp-content/uploads/2024/07/ir_2024_1877.pdf</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/subte-estaciones</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>sin licencia declarada (publicación oficial; citar fuente)</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>declarado</t>
+          <t>vivo</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1640,17 +1640,17 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>2022</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>poblacion_comunas=3.121.707 habitantes (Censo 2022 definitivo. suma de comunas)</t>
+          <t>estaciones_distintas=88 estaciones (nombres distintos); estaciones_linea=90 pares estación-línea; lineas=6 líneas</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Solo población por comuna. Faltan viviendas, hogares y servicios por comuna (informe 1877 los trae en gráficos) y radios censales</t>
+          <t>Accesibilidad; campo línea (A, B, C…) en subte_lineas.geojson. Viajes por estación: ver ba_subte_molinetes</t>
         </is>
       </c>
     </row>
@@ -1660,27 +1660,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>eoh_caba</t>
+          <t>ba_subte_molinetes</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Encuesta de Ocupación Hotelera y Parahotelera (EOH), INDEC y Subsecretaría de Turismo</t>
+          <t>Subte: Viajes Molinetes.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>turismo</t>
+          <t>correlaciones, subte_molinetes</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://datos.yvera.gob.ar/dataset/encuesta-ocupacion-hotelera-parahotelera-eoh</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/subte-viajes-molinetes</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1695,17 +1695,17 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>2024, 2025-08</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>ocupacion_plazas_ultimo_mes=39.0 % de plazas ocupadas (hoteles y parahoteles); pernoctaciones_ultimo_mes=660.646 pernoctaciones (noches) por mes; viajeros_2024=3.993.697 viajeros hospedados en el año; viajeros_no_residentes_ultimo_mes=136.364 viajeros no residentes hospedados por mes; viajeros_residentes_ultimo_mes=173.564 viajeros residentes hospedados por mes; viajeros_total_ultimo_mes=309.928 viajeros hospedados por mes</t>
+          <t>lineas=7 líneas (incluye Premetro PM); meses_con_datos_2025=12 meses; pasajeros_subte_2025=206.459.041 pasajeros (validaciones en molinetes. líneas A-H)</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Tarifa media, estadía media y ocupación por categoría; se publica con ~1 año de rezago</t>
+          <t>Franja horaria (cada 15 min) y años anteriores sin cargar; se guarda solo el agregado por estación y mes</t>
         </is>
       </c>
     </row>
@@ -1715,27 +1715,27 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>wikimedia_pageviews</t>
+          <t>ba_tejido_urbano</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Wikimedia Pageviews API</t>
+          <t>Tejido Urbano</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>escucha</t>
+          <t>correlaciones, edificios</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://wikimedia.org/api/rest_v1/metrics/pageviews/per-article/es.wikipedia/all-access/user/Buenos_Aires/monthly/20250101/20260831</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/tejido-urbano</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>CC0</t>
+          <t>CC-BY-2.5-AR</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1750,17 +1750,17 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>vistas_ultimo_mes=36.339 vistas de personas</t>
+          <t>altura_maxima=221.4 m (volumen más alto del tejido); altura_mediana_parcela=5.6 m (mediana de la altura máxima por parcela); parcelas_edificadas=309.164 parcelas edificadas; volumenes_descartados=2 volúmenes con altura 0 o mayor a 250 m (errores); volumenes_edificados=1.386.616 volúmenes edificados (filas del tejido)</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Otros artículos/idiomas; mide interés, no opinión ni sentimiento</t>
+          <t>Superficie de cada volumen (para m³ construidos) y geometrías 3D (~1 GB: GeoParquet/PMTiles, ver contrato); datos hasta 2021</t>
         </is>
       </c>
     </row>
@@ -1768,20 +1768,24 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>ba_tmi</t>
+        </is>
+      </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Información Censal por Radio (BA Data)</t>
+          <t>Información Meteorológica</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>(demografía 2022 por barrio)</t>
+          <t>sensores</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-censal-por-radio</t>
+          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-meteorologica</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1791,15 +1795,27 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>insuficiente</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr"/>
-      <c r="I25" s="2" t="inlineStr"/>
-      <c r="J25" s="2" t="inlineStr"/>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>ba_tmi=16 torres de monitoreo inteligente</t>
+        </is>
+      </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Solo radios de 2001 y 2010: no da población 2022 por barrio. Los radios 2022 no están en BA Data</t>
+          <t>Lecturas meteorológicas de las torres (temperatura, humedad); aquí solo inventario de 16 torres</t>
         </is>
       </c>
     </row>
@@ -1807,30 +1823,54 @@
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>dgeyc_censo2022</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>BA Data reclamos 147</t>
+          <t>Censo Nacional 2022, resultados definitivos CABA (INDEC; DGEyC GCBA, informe 1877)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>(reclamos)</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
+          <t>demografia</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.estadisticaciudad.gob.ar/eyc/wp-content/uploads/2024/07/ir_2024_1877.pdf</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>sin licencia declarada (publicación oficial; citar fuente)</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>descartado</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
+          <t>declarado</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>poblacion_comunas=3.121.707 habitantes (Censo 2022 definitivo. suma de comunas)</t>
+        </is>
+      </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Descartado por descarga pesada; faltan todos los campos</t>
+          <t>Solo población por comuna. Faltan viviendas, hogares y servicios por comuna (informe 1877 los trae en gráficos) y radios censales</t>
         </is>
       </c>
     </row>
@@ -1838,28 +1878,373 @@
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>eoh_caba</t>
+        </is>
+      </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
+          <t>Encuesta de Ocupación Hotelera y Parahotelera (EOH), INDEC y Subsecretaría de Turismo</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>turismo</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://datos.yvera.gob.ar/dataset/encuesta-ocupacion-hotelera-parahotelera-eoh</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>2024, 2025-08</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>ocupacion_plazas_ultimo_mes=39.0 % de plazas ocupadas (hoteles y parahoteles); pernoctaciones_ultimo_mes=660.646 pernoctaciones (noches) por mes; viajeros_2024=3.993.697 viajeros hospedados en el año; viajeros_no_residentes_ultimo_mes=136.364 viajeros no residentes hospedados por mes; viajeros_residentes_ultimo_mes=173.564 viajeros residentes hospedados por mes; viajeros_total_ultimo_mes=309.928 viajeros hospedados por mes</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Tarifa media, estadía media y ocupación por categoría; se publica con ~1 año de rezago</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>ipcba</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Índice de Precios al Consumidor de la Ciudad de Buenos Aires (IPCBA), Estadística Ciudad; republicado por la Subsecretaría de Programación Macroeconómica</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>economia, municipio</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.estadisticaciudad.gob.ar/eyc/?cat=93</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>2025, 2026-08</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>inflacion_2025=31.8 % de variación del IPCBA diciembre a diciembre; inflacion_interanual=33.3 % de variación del IPCBA 2025-08 → 2026-08; ipcba_promedio_2025=1.896.37 índice IPCBA promedio del año; ipcba_ultimo_mes=2.596.6 índice IPCBA nivel general</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Divisiones del IPCBA (alimentos, vivienda, transporte…); serie desde 2022-02 (base 2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>open_meteo</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Open-Meteo Historical Weather API (reanálisis ERA5/ERA5-Land, ECMWF)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>clima</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://open-meteo.com/en/docs/historical-weather-api</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>dias_32c_2025=28 días con máxima ≥ 32 °C; maxima_2025=38.7 °C (máxima diaria más alta del año); precipitacion_2025=1.233 mm (total anual); temperatura_media_2025=18.4 °C (media anual)</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>Viento, humedad y radiación; dato de grilla (no estación, no distingue barrios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>sipa_caba</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Asalariados registrados del sector privado por provincia (SIPA), Ministerio de Economía</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>economia</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.economia.gob.ar/datos/</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>asalariados_privados_ultimo_mes=1.485.000 asalariados registrados del sector privado (sin estacionalidad)</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>Por rama de actividad y salario medio; empleo público y no registrado no incluidos</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>wikimedia_pageviews</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Wikimedia Pageviews API</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>escucha</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://wikimedia.org/api/rest_v1/metrics/pageviews/per-article/es.wikipedia/all-access/user/Buenos_Aires/monthly/20250101/20260831</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>CC0</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>vivo</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>vistas_ultimo_mes=36.339 vistas de personas</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Otros artículos/idiomas; mide interés, no opinión ni sentimiento</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Información Censal por Radio (BA Data)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>(demografía 2022 por barrio)</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://data.buenosaires.gob.ar/km/dataset/informacion-censal-por-radio</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>CC-BY-2.5-AR</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>insuficiente</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Solo radios de 2001 y 2010: no da población 2022 por barrio. Los radios 2022 no están en BA Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>BA Data reclamos 147</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>(reclamos)</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>descartado</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Descartado por descarga pesada; faltan todos los campos</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
           <t>API de transporte/sensores</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>(sensores en tiempo real)</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>pendiente</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr"/>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>Requiere credenciales; faltan lecturas, frecuencia y licencia</t>
         </is>

</xml_diff>

<commit_message>
Entrega 1: diccionario de datos lleno desde el lago (40 fuentes, 161 campos, bitácora IA); sensores en vivo: API suspendida
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fuentes_gemelo_buenos_aires.xlsx
+++ b/fuentes_gemelo_buenos_aires.xlsx
@@ -1595,7 +1595,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Lecturas en vivo (API de transporte con credenciales); aquí solo inventario de 52 sensores</t>
+          <t>Lecturas en vivo (API de Transporte, suspendida por el portal); aquí solo inventario de 52 sensores</t>
         </is>
       </c>
     </row>
@@ -2246,7 +2246,7 @@
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Requiere credenciales; faltan lecturas, frecuencia y licencia</t>
+          <t>El portal suspendió las API y GTFS (aviso del 2026-10-06); faltan lecturas</t>
         </is>
       </c>
     </row>

</xml_diff>